<commit_message>
Fix overtime hours dropped when the day isn't marked as attended
jamLembur (overtime) was only summed for days where hadir=true, so
overtime worked on a day off (e.g. Sunday, where an employee comes in
just for overtime without a regular attendance mark) was silently
excluded from the weekly payroll total. Overtime should count for
every day in the pay period regardless of the attendance flag — only
"hari hadir" (days present) should depend on it.

Fixes both the website (www/app.js computePayrollFromAbsensi) and the
Excel workbook's Penggajian sheet (Jam Lembur SUMIFS no longer
requires Hadir="Ya").
</commit_message>
<xml_diff>
--- a/excel/MitraCreative_Keuangan.xlsx
+++ b/excel/MitraCreative_Keuangan.xlsx
@@ -1996,11 +1996,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="16073785"/>
-        <c:axId val="18403217"/>
+        <c:axId val="68840019"/>
+        <c:axId val="81768836"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="16073785"/>
+        <c:axId val="68840019"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2032,7 +2032,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18403217"/>
+        <c:crossAx val="81768836"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2040,7 +2040,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="18403217"/>
+        <c:axId val="81768836"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2116,7 +2116,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16073785"/>
+        <c:crossAx val="68840019"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2407,11 +2407,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="28996327"/>
-        <c:axId val="17459093"/>
+        <c:axId val="36340200"/>
+        <c:axId val="20369396"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="28996327"/>
+        <c:axId val="36340200"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2443,7 +2443,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17459093"/>
+        <c:crossAx val="20369396"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2451,7 +2451,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="17459093"/>
+        <c:axId val="20369396"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2493,7 +2493,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="28996327"/>
+        <c:crossAx val="36340200"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -26498,7 +26498,7 @@
         <v/>
       </c>
       <c r="J3" s="12" t="str">
-        <f aca="false">IF(B3="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B3,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E3,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F3,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B3="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B3,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E3,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F3))</f>
         <v/>
       </c>
       <c r="K3" s="12" t="str">
@@ -26572,7 +26572,7 @@
         <v/>
       </c>
       <c r="J4" s="12" t="str">
-        <f aca="false">IF(B4="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B4,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E4,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F4,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B4="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B4,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E4,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F4))</f>
         <v/>
       </c>
       <c r="K4" s="12" t="str">
@@ -26646,7 +26646,7 @@
         <v/>
       </c>
       <c r="J5" s="12" t="str">
-        <f aca="false">IF(B5="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B5,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E5,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F5,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B5="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B5,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E5,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F5))</f>
         <v/>
       </c>
       <c r="K5" s="12" t="str">
@@ -26720,7 +26720,7 @@
         <v/>
       </c>
       <c r="J6" s="12" t="str">
-        <f aca="false">IF(B6="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B6,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E6,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F6,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B6="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B6,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E6,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F6))</f>
         <v/>
       </c>
       <c r="K6" s="12" t="str">
@@ -26794,7 +26794,7 @@
         <v/>
       </c>
       <c r="J7" s="12" t="str">
-        <f aca="false">IF(B7="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B7,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E7,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F7,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B7="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B7,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E7,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F7))</f>
         <v/>
       </c>
       <c r="K7" s="12" t="str">
@@ -26868,7 +26868,7 @@
         <v/>
       </c>
       <c r="J8" s="12" t="str">
-        <f aca="false">IF(B8="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B8,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E8,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F8,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B8="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B8,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E8,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F8))</f>
         <v/>
       </c>
       <c r="K8" s="12" t="str">
@@ -26942,7 +26942,7 @@
         <v/>
       </c>
       <c r="J9" s="12" t="str">
-        <f aca="false">IF(B9="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B9,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E9,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F9,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B9="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B9,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E9,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F9))</f>
         <v/>
       </c>
       <c r="K9" s="12" t="str">
@@ -27016,7 +27016,7 @@
         <v/>
       </c>
       <c r="J10" s="12" t="str">
-        <f aca="false">IF(B10="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B10,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E10,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F10,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B10="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B10,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E10,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F10))</f>
         <v/>
       </c>
       <c r="K10" s="12" t="str">
@@ -27090,7 +27090,7 @@
         <v/>
       </c>
       <c r="J11" s="12" t="str">
-        <f aca="false">IF(B11="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B11,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E11,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F11,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B11="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B11,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E11,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F11))</f>
         <v/>
       </c>
       <c r="K11" s="12" t="str">
@@ -27164,7 +27164,7 @@
         <v/>
       </c>
       <c r="J12" s="12" t="str">
-        <f aca="false">IF(B12="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B12,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E12,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F12,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B12="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B12,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E12,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F12))</f>
         <v/>
       </c>
       <c r="K12" s="12" t="str">
@@ -27238,7 +27238,7 @@
         <v/>
       </c>
       <c r="J13" s="12" t="str">
-        <f aca="false">IF(B13="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B13,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E13,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F13,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B13="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B13,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E13,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F13))</f>
         <v/>
       </c>
       <c r="K13" s="12" t="str">
@@ -27312,7 +27312,7 @@
         <v/>
       </c>
       <c r="J14" s="12" t="str">
-        <f aca="false">IF(B14="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B14,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E14,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F14,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B14="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B14,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E14,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F14))</f>
         <v/>
       </c>
       <c r="K14" s="12" t="str">
@@ -27386,7 +27386,7 @@
         <v/>
       </c>
       <c r="J15" s="12" t="str">
-        <f aca="false">IF(B15="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B15,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E15,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F15,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B15="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B15,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E15,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F15))</f>
         <v/>
       </c>
       <c r="K15" s="12" t="str">
@@ -27460,7 +27460,7 @@
         <v/>
       </c>
       <c r="J16" s="12" t="str">
-        <f aca="false">IF(B16="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B16,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E16,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F16,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B16="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B16,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E16,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F16))</f>
         <v/>
       </c>
       <c r="K16" s="12" t="str">
@@ -27534,7 +27534,7 @@
         <v/>
       </c>
       <c r="J17" s="12" t="str">
-        <f aca="false">IF(B17="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B17,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E17,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F17,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B17="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B17,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E17,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F17))</f>
         <v/>
       </c>
       <c r="K17" s="12" t="str">
@@ -27608,7 +27608,7 @@
         <v/>
       </c>
       <c r="J18" s="12" t="str">
-        <f aca="false">IF(B18="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B18,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E18,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F18,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B18="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B18,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E18,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F18))</f>
         <v/>
       </c>
       <c r="K18" s="12" t="str">
@@ -27682,7 +27682,7 @@
         <v/>
       </c>
       <c r="J19" s="12" t="str">
-        <f aca="false">IF(B19="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B19,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E19,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F19,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B19="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B19,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E19,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F19))</f>
         <v/>
       </c>
       <c r="K19" s="12" t="str">
@@ -27756,7 +27756,7 @@
         <v/>
       </c>
       <c r="J20" s="12" t="str">
-        <f aca="false">IF(B20="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B20,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E20,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F20,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B20="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B20,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E20,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F20))</f>
         <v/>
       </c>
       <c r="K20" s="12" t="str">
@@ -27830,7 +27830,7 @@
         <v/>
       </c>
       <c r="J21" s="12" t="str">
-        <f aca="false">IF(B21="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B21,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E21,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F21,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B21="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B21,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E21,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F21))</f>
         <v/>
       </c>
       <c r="K21" s="12" t="str">
@@ -27904,7 +27904,7 @@
         <v/>
       </c>
       <c r="J22" s="12" t="str">
-        <f aca="false">IF(B22="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B22,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E22,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F22,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B22="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B22,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E22,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F22))</f>
         <v/>
       </c>
       <c r="K22" s="12" t="str">
@@ -27978,7 +27978,7 @@
         <v/>
       </c>
       <c r="J23" s="12" t="str">
-        <f aca="false">IF(B23="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B23,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E23,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F23,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B23="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B23,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E23,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F23))</f>
         <v/>
       </c>
       <c r="K23" s="12" t="str">
@@ -28052,7 +28052,7 @@
         <v/>
       </c>
       <c r="J24" s="12" t="str">
-        <f aca="false">IF(B24="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B24,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E24,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F24,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B24="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B24,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E24,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F24))</f>
         <v/>
       </c>
       <c r="K24" s="12" t="str">
@@ -28126,7 +28126,7 @@
         <v/>
       </c>
       <c r="J25" s="12" t="str">
-        <f aca="false">IF(B25="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B25,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E25,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F25,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B25="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B25,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E25,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F25))</f>
         <v/>
       </c>
       <c r="K25" s="12" t="str">
@@ -28200,7 +28200,7 @@
         <v/>
       </c>
       <c r="J26" s="12" t="str">
-        <f aca="false">IF(B26="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B26,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E26,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F26,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B26="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B26,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E26,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F26))</f>
         <v/>
       </c>
       <c r="K26" s="12" t="str">
@@ -28274,7 +28274,7 @@
         <v/>
       </c>
       <c r="J27" s="12" t="str">
-        <f aca="false">IF(B27="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B27,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E27,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F27,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B27="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B27,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E27,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F27))</f>
         <v/>
       </c>
       <c r="K27" s="12" t="str">
@@ -28348,7 +28348,7 @@
         <v/>
       </c>
       <c r="J28" s="12" t="str">
-        <f aca="false">IF(B28="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B28,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E28,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F28,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B28="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B28,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E28,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F28))</f>
         <v/>
       </c>
       <c r="K28" s="12" t="str">
@@ -28422,7 +28422,7 @@
         <v/>
       </c>
       <c r="J29" s="12" t="str">
-        <f aca="false">IF(B29="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B29,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E29,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F29,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B29="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B29,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E29,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F29))</f>
         <v/>
       </c>
       <c r="K29" s="12" t="str">
@@ -28496,7 +28496,7 @@
         <v/>
       </c>
       <c r="J30" s="12" t="str">
-        <f aca="false">IF(B30="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B30,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E30,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F30,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B30="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B30,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E30,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F30))</f>
         <v/>
       </c>
       <c r="K30" s="12" t="str">
@@ -28570,7 +28570,7 @@
         <v/>
       </c>
       <c r="J31" s="12" t="str">
-        <f aca="false">IF(B31="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B31,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E31,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F31,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B31="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B31,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E31,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F31))</f>
         <v/>
       </c>
       <c r="K31" s="12" t="str">
@@ -28644,7 +28644,7 @@
         <v/>
       </c>
       <c r="J32" s="12" t="str">
-        <f aca="false">IF(B32="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B32,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E32,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F32,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B32="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B32,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E32,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F32))</f>
         <v/>
       </c>
       <c r="K32" s="12" t="str">
@@ -28718,7 +28718,7 @@
         <v/>
       </c>
       <c r="J33" s="12" t="str">
-        <f aca="false">IF(B33="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B33,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E33,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F33,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B33="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B33,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E33,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F33))</f>
         <v/>
       </c>
       <c r="K33" s="12" t="str">
@@ -28792,7 +28792,7 @@
         <v/>
       </c>
       <c r="J34" s="12" t="str">
-        <f aca="false">IF(B34="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B34,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E34,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F34,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B34="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B34,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E34,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F34))</f>
         <v/>
       </c>
       <c r="K34" s="12" t="str">
@@ -28866,7 +28866,7 @@
         <v/>
       </c>
       <c r="J35" s="12" t="str">
-        <f aca="false">IF(B35="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B35,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E35,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F35,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B35="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B35,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E35,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F35))</f>
         <v/>
       </c>
       <c r="K35" s="12" t="str">
@@ -28940,7 +28940,7 @@
         <v/>
       </c>
       <c r="J36" s="12" t="str">
-        <f aca="false">IF(B36="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B36,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E36,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F36,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B36="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B36,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E36,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F36))</f>
         <v/>
       </c>
       <c r="K36" s="12" t="str">
@@ -29014,7 +29014,7 @@
         <v/>
       </c>
       <c r="J37" s="12" t="str">
-        <f aca="false">IF(B37="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B37,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E37,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F37,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B37="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B37,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E37,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F37))</f>
         <v/>
       </c>
       <c r="K37" s="12" t="str">
@@ -29088,7 +29088,7 @@
         <v/>
       </c>
       <c r="J38" s="12" t="str">
-        <f aca="false">IF(B38="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B38,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E38,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F38,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B38="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B38,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E38,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F38))</f>
         <v/>
       </c>
       <c r="K38" s="12" t="str">
@@ -29162,7 +29162,7 @@
         <v/>
       </c>
       <c r="J39" s="12" t="str">
-        <f aca="false">IF(B39="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B39,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E39,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F39,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B39="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B39,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E39,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F39))</f>
         <v/>
       </c>
       <c r="K39" s="12" t="str">
@@ -29236,7 +29236,7 @@
         <v/>
       </c>
       <c r="J40" s="12" t="str">
-        <f aca="false">IF(B40="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B40,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E40,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F40,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B40="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B40,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E40,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F40))</f>
         <v/>
       </c>
       <c r="K40" s="12" t="str">
@@ -29310,7 +29310,7 @@
         <v/>
       </c>
       <c r="J41" s="12" t="str">
-        <f aca="false">IF(B41="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B41,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E41,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F41,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B41="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B41,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E41,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F41))</f>
         <v/>
       </c>
       <c r="K41" s="12" t="str">
@@ -29384,7 +29384,7 @@
         <v/>
       </c>
       <c r="J42" s="12" t="str">
-        <f aca="false">IF(B42="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B42,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E42,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F42,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B42="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B42,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E42,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F42))</f>
         <v/>
       </c>
       <c r="K42" s="12" t="str">
@@ -29458,7 +29458,7 @@
         <v/>
       </c>
       <c r="J43" s="12" t="str">
-        <f aca="false">IF(B43="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B43,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E43,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F43,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B43="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B43,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E43,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F43))</f>
         <v/>
       </c>
       <c r="K43" s="12" t="str">
@@ -29532,7 +29532,7 @@
         <v/>
       </c>
       <c r="J44" s="12" t="str">
-        <f aca="false">IF(B44="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B44,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E44,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F44,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B44="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B44,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E44,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F44))</f>
         <v/>
       </c>
       <c r="K44" s="12" t="str">
@@ -29606,7 +29606,7 @@
         <v/>
       </c>
       <c r="J45" s="12" t="str">
-        <f aca="false">IF(B45="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B45,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E45,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F45,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B45="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B45,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E45,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F45))</f>
         <v/>
       </c>
       <c r="K45" s="12" t="str">
@@ -29680,7 +29680,7 @@
         <v/>
       </c>
       <c r="J46" s="12" t="str">
-        <f aca="false">IF(B46="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B46,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E46,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F46,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B46="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B46,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E46,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F46))</f>
         <v/>
       </c>
       <c r="K46" s="12" t="str">
@@ -29754,7 +29754,7 @@
         <v/>
       </c>
       <c r="J47" s="12" t="str">
-        <f aca="false">IF(B47="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B47,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E47,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F47,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B47="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B47,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E47,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F47))</f>
         <v/>
       </c>
       <c r="K47" s="12" t="str">
@@ -29828,7 +29828,7 @@
         <v/>
       </c>
       <c r="J48" s="12" t="str">
-        <f aca="false">IF(B48="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B48,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E48,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F48,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B48="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B48,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E48,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F48))</f>
         <v/>
       </c>
       <c r="K48" s="12" t="str">
@@ -29902,7 +29902,7 @@
         <v/>
       </c>
       <c r="J49" s="12" t="str">
-        <f aca="false">IF(B49="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B49,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E49,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F49,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B49="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B49,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E49,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F49))</f>
         <v/>
       </c>
       <c r="K49" s="12" t="str">
@@ -29976,7 +29976,7 @@
         <v/>
       </c>
       <c r="J50" s="12" t="str">
-        <f aca="false">IF(B50="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B50,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E50,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F50,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B50="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B50,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E50,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F50))</f>
         <v/>
       </c>
       <c r="K50" s="12" t="str">
@@ -30050,7 +30050,7 @@
         <v/>
       </c>
       <c r="J51" s="12" t="str">
-        <f aca="false">IF(B51="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B51,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E51,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F51,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B51="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B51,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E51,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F51))</f>
         <v/>
       </c>
       <c r="K51" s="12" t="str">
@@ -30124,7 +30124,7 @@
         <v/>
       </c>
       <c r="J52" s="12" t="str">
-        <f aca="false">IF(B52="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B52,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E52,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F52,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B52="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B52,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E52,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F52))</f>
         <v/>
       </c>
       <c r="K52" s="12" t="str">
@@ -30198,7 +30198,7 @@
         <v/>
       </c>
       <c r="J53" s="12" t="str">
-        <f aca="false">IF(B53="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B53,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E53,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F53,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B53="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B53,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E53,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F53))</f>
         <v/>
       </c>
       <c r="K53" s="12" t="str">
@@ -30272,7 +30272,7 @@
         <v/>
       </c>
       <c r="J54" s="12" t="str">
-        <f aca="false">IF(B54="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B54,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E54,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F54,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B54="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B54,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E54,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F54))</f>
         <v/>
       </c>
       <c r="K54" s="12" t="str">
@@ -30346,7 +30346,7 @@
         <v/>
       </c>
       <c r="J55" s="12" t="str">
-        <f aca="false">IF(B55="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B55,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E55,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F55,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B55="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B55,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E55,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F55))</f>
         <v/>
       </c>
       <c r="K55" s="12" t="str">
@@ -30420,7 +30420,7 @@
         <v/>
       </c>
       <c r="J56" s="12" t="str">
-        <f aca="false">IF(B56="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B56,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E56,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F56,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B56="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B56,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E56,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F56))</f>
         <v/>
       </c>
       <c r="K56" s="12" t="str">
@@ -30494,7 +30494,7 @@
         <v/>
       </c>
       <c r="J57" s="12" t="str">
-        <f aca="false">IF(B57="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B57,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E57,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F57,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B57="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B57,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E57,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F57))</f>
         <v/>
       </c>
       <c r="K57" s="12" t="str">
@@ -30568,7 +30568,7 @@
         <v/>
       </c>
       <c r="J58" s="12" t="str">
-        <f aca="false">IF(B58="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B58,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E58,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F58,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B58="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B58,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E58,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F58))</f>
         <v/>
       </c>
       <c r="K58" s="12" t="str">
@@ -30642,7 +30642,7 @@
         <v/>
       </c>
       <c r="J59" s="12" t="str">
-        <f aca="false">IF(B59="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B59,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E59,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F59,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B59="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B59,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E59,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F59))</f>
         <v/>
       </c>
       <c r="K59" s="12" t="str">
@@ -30716,7 +30716,7 @@
         <v/>
       </c>
       <c r="J60" s="12" t="str">
-        <f aca="false">IF(B60="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B60,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E60,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F60,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B60="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B60,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E60,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F60))</f>
         <v/>
       </c>
       <c r="K60" s="12" t="str">
@@ -30790,7 +30790,7 @@
         <v/>
       </c>
       <c r="J61" s="12" t="str">
-        <f aca="false">IF(B61="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B61,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E61,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F61,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B61="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B61,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E61,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F61))</f>
         <v/>
       </c>
       <c r="K61" s="12" t="str">
@@ -30864,7 +30864,7 @@
         <v/>
       </c>
       <c r="J62" s="12" t="str">
-        <f aca="false">IF(B62="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B62,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E62,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F62,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B62="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B62,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E62,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F62))</f>
         <v/>
       </c>
       <c r="K62" s="12" t="str">
@@ -30938,7 +30938,7 @@
         <v/>
       </c>
       <c r="J63" s="12" t="str">
-        <f aca="false">IF(B63="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B63,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E63,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F63,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B63="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B63,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E63,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F63))</f>
         <v/>
       </c>
       <c r="K63" s="12" t="str">
@@ -31012,7 +31012,7 @@
         <v/>
       </c>
       <c r="J64" s="12" t="str">
-        <f aca="false">IF(B64="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B64,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E64,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F64,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B64="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B64,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E64,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F64))</f>
         <v/>
       </c>
       <c r="K64" s="12" t="str">
@@ -31086,7 +31086,7 @@
         <v/>
       </c>
       <c r="J65" s="12" t="str">
-        <f aca="false">IF(B65="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B65,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E65,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F65,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B65="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B65,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E65,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F65))</f>
         <v/>
       </c>
       <c r="K65" s="12" t="str">
@@ -31160,7 +31160,7 @@
         <v/>
       </c>
       <c r="J66" s="12" t="str">
-        <f aca="false">IF(B66="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B66,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E66,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F66,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B66="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B66,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E66,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F66))</f>
         <v/>
       </c>
       <c r="K66" s="12" t="str">
@@ -31234,7 +31234,7 @@
         <v/>
       </c>
       <c r="J67" s="12" t="str">
-        <f aca="false">IF(B67="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B67,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E67,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F67,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B67="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B67,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E67,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F67))</f>
         <v/>
       </c>
       <c r="K67" s="12" t="str">
@@ -31308,7 +31308,7 @@
         <v/>
       </c>
       <c r="J68" s="12" t="str">
-        <f aca="false">IF(B68="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B68,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E68,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F68,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B68="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B68,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E68,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F68))</f>
         <v/>
       </c>
       <c r="K68" s="12" t="str">
@@ -31382,7 +31382,7 @@
         <v/>
       </c>
       <c r="J69" s="12" t="str">
-        <f aca="false">IF(B69="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B69,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E69,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F69,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B69="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B69,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E69,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F69))</f>
         <v/>
       </c>
       <c r="K69" s="12" t="str">
@@ -31456,7 +31456,7 @@
         <v/>
       </c>
       <c r="J70" s="12" t="str">
-        <f aca="false">IF(B70="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B70,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E70,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F70,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B70="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B70,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E70,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F70))</f>
         <v/>
       </c>
       <c r="K70" s="12" t="str">
@@ -31530,7 +31530,7 @@
         <v/>
       </c>
       <c r="J71" s="12" t="str">
-        <f aca="false">IF(B71="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B71,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E71,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F71,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B71="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B71,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E71,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F71))</f>
         <v/>
       </c>
       <c r="K71" s="12" t="str">
@@ -31604,7 +31604,7 @@
         <v/>
       </c>
       <c r="J72" s="12" t="str">
-        <f aca="false">IF(B72="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B72,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E72,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F72,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B72="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B72,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E72,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F72))</f>
         <v/>
       </c>
       <c r="K72" s="12" t="str">
@@ -31678,7 +31678,7 @@
         <v/>
       </c>
       <c r="J73" s="12" t="str">
-        <f aca="false">IF(B73="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B73,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E73,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F73,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B73="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B73,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E73,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F73))</f>
         <v/>
       </c>
       <c r="K73" s="12" t="str">
@@ -31752,7 +31752,7 @@
         <v/>
       </c>
       <c r="J74" s="12" t="str">
-        <f aca="false">IF(B74="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B74,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E74,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F74,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B74="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B74,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E74,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F74))</f>
         <v/>
       </c>
       <c r="K74" s="12" t="str">
@@ -31826,7 +31826,7 @@
         <v/>
       </c>
       <c r="J75" s="12" t="str">
-        <f aca="false">IF(B75="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B75,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E75,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F75,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B75="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B75,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E75,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F75))</f>
         <v/>
       </c>
       <c r="K75" s="12" t="str">
@@ -31900,7 +31900,7 @@
         <v/>
       </c>
       <c r="J76" s="12" t="str">
-        <f aca="false">IF(B76="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B76,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E76,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F76,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B76="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B76,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E76,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F76))</f>
         <v/>
       </c>
       <c r="K76" s="12" t="str">
@@ -31974,7 +31974,7 @@
         <v/>
       </c>
       <c r="J77" s="12" t="str">
-        <f aca="false">IF(B77="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B77,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E77,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F77,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B77="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B77,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E77,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F77))</f>
         <v/>
       </c>
       <c r="K77" s="12" t="str">
@@ -32048,7 +32048,7 @@
         <v/>
       </c>
       <c r="J78" s="12" t="str">
-        <f aca="false">IF(B78="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B78,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E78,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F78,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B78="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B78,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E78,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F78))</f>
         <v/>
       </c>
       <c r="K78" s="12" t="str">
@@ -32122,7 +32122,7 @@
         <v/>
       </c>
       <c r="J79" s="12" t="str">
-        <f aca="false">IF(B79="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B79,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E79,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F79,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B79="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B79,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E79,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F79))</f>
         <v/>
       </c>
       <c r="K79" s="12" t="str">
@@ -32196,7 +32196,7 @@
         <v/>
       </c>
       <c r="J80" s="12" t="str">
-        <f aca="false">IF(B80="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B80,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E80,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F80,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B80="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B80,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E80,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F80))</f>
         <v/>
       </c>
       <c r="K80" s="12" t="str">
@@ -32270,7 +32270,7 @@
         <v/>
       </c>
       <c r="J81" s="12" t="str">
-        <f aca="false">IF(B81="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B81,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E81,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F81,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B81="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B81,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E81,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F81))</f>
         <v/>
       </c>
       <c r="K81" s="12" t="str">
@@ -32344,7 +32344,7 @@
         <v/>
       </c>
       <c r="J82" s="12" t="str">
-        <f aca="false">IF(B82="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B82,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E82,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F82,'Absensi Harian'!$C$4:$C$153,"Ya"))</f>
+        <f aca="false">IF(B82="","",SUMIFS('Absensi Harian'!$D$4:$D$153,'Absensi Harian'!$B$4:$B$153,B82,'Absensi Harian'!$A$4:$A$153,"&gt;="&amp;E82,'Absensi Harian'!$A$4:$A$153,"&lt;="&amp;F82))</f>
         <v/>
       </c>
       <c r="K82" s="12" t="str">

</xml_diff>